<commit_message>
Implemented method to calculate N2O from organic soils
</commit_message>
<xml_diff>
--- a/data/prod_parameters/PlantNutrientMgmt.xlsx
+++ b/data/prod_parameters/PlantNutrientMgmt.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1054" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1058" uniqueCount="192">
   <si>
     <t>f_crop</t>
   </si>
@@ -614,6 +614,12 @@
   </si>
   <si>
     <t>emission factors are available for different spreading techniques and timings. Use these!!!</t>
+  </si>
+  <si>
+    <t>soil_losses_organic_soils</t>
+  </si>
+  <si>
+    <t>kg N2O-N/ha</t>
   </si>
 </sst>
 </file>
@@ -1013,7 +1019,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R292"/>
+  <dimension ref="A1:R294"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="1"/>
@@ -5923,6 +5929,9 @@
       </c>
     </row>
     <row r="291" spans="6:15" x14ac:dyDescent="0.25">
+      <c r="J291" t="s">
+        <v>171</v>
+      </c>
       <c r="K291" t="s">
         <v>184</v>
       </c>
@@ -5957,6 +5966,20 @@
       </c>
       <c r="O292" t="s">
         <v>174</v>
+      </c>
+    </row>
+    <row r="294" spans="6:15" x14ac:dyDescent="0.25">
+      <c r="J294" t="s">
+        <v>171</v>
+      </c>
+      <c r="K294" t="s">
+        <v>190</v>
+      </c>
+      <c r="L294">
+        <v>13</v>
+      </c>
+      <c r="M294" t="s">
+        <v>191</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implemented way to handle specifying filters on aggregate level in Excel sheets without need to change in the code
</commit_message>
<xml_diff>
--- a/data/prod_parameters/PlantNutrientMgmt.xlsx
+++ b/data/prod_parameters/PlantNutrientMgmt.xlsx
@@ -322,9 +322,6 @@
     <t>po8</t>
   </si>
   <si>
-    <t>f_po8</t>
-  </si>
-  <si>
     <t>Höstvete foder/bröd, södra götaland</t>
   </si>
   <si>
@@ -620,6 +617,9 @@
   </si>
   <si>
     <t>kg N2O-N/ha</t>
+  </si>
+  <si>
+    <t>f_po8:region</t>
   </si>
 </sst>
 </file>
@@ -1041,7 +1041,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>100</v>
+        <v>191</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>90</v>
@@ -1050,22 +1050,22 @@
         <v>8</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="I1" s="1" t="s">
-        <v>140</v>
-      </c>
       <c r="J1" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>1</v>
@@ -1085,7 +1085,7 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
@@ -1104,44 +1104,44 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="K4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="L4">
         <v>91</v>
       </c>
       <c r="M4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="N4" t="s">
+        <v>121</v>
+      </c>
+      <c r="O4" t="s">
         <v>122</v>
-      </c>
-      <c r="O4" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="K5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="L5">
         <v>22</v>
       </c>
       <c r="M5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="N5" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="O5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B7" s="2"/>
       <c r="C7" s="2"/>
@@ -1160,87 +1160,87 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C8" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="K8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="L8">
         <v>0</v>
       </c>
       <c r="M8" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="N8" s="5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C9" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E9" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K9" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="L9">
         <v>59</v>
       </c>
       <c r="M9" t="s">
+        <v>127</v>
+      </c>
+      <c r="N9" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="O9" t="s">
         <v>128</v>
-      </c>
-      <c r="N9" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="O9" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C10" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="K10" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="L10">
         <v>7</v>
       </c>
       <c r="M10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="O10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C11" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E11" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="K11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="L11">
         <v>34</v>
       </c>
       <c r="M11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="O11" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -1304,7 +1304,7 @@
         <v>-0.80359999999999998</v>
       </c>
       <c r="N17" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
@@ -1357,7 +1357,7 @@
         <v>-0.71430000000000005</v>
       </c>
       <c r="N21" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
@@ -1544,7 +1544,7 @@
         <v>-1.25</v>
       </c>
       <c r="N34" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
@@ -1668,7 +1668,7 @@
         <v>-0.71430000000000005</v>
       </c>
       <c r="N42" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
@@ -1843,7 +1843,7 @@
         <v>-1.25</v>
       </c>
       <c r="N54" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.25">
@@ -1891,7 +1891,7 @@
         <v>-2E-12</v>
       </c>
       <c r="N57" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.25">
@@ -2049,7 +2049,7 @@
         <v>0</v>
       </c>
       <c r="N66" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.25">
@@ -2295,7 +2295,7 @@
         <v>-1.25</v>
       </c>
       <c r="N81" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="82" spans="1:14" x14ac:dyDescent="0.25">
@@ -2771,7 +2771,7 @@
         <v>-2.5000000000000001E-2</v>
       </c>
       <c r="N113" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="114" spans="1:14" x14ac:dyDescent="0.25">
@@ -3145,7 +3145,7 @@
         <v>1.3846000000000001</v>
       </c>
       <c r="N137" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="138" spans="1:15" x14ac:dyDescent="0.25">
@@ -3389,7 +3389,7 @@
         <v>3.3332999999999999</v>
       </c>
       <c r="N149" s="7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="150" spans="1:15" x14ac:dyDescent="0.25">
@@ -3527,7 +3527,7 @@
         <v>100</v>
       </c>
       <c r="N157" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="158" spans="1:15" x14ac:dyDescent="0.25">
@@ -3671,7 +3671,7 @@
     </row>
     <row r="170" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A170" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B170" s="2"/>
       <c r="C170" s="2"/>
@@ -4743,7 +4743,7 @@
     </row>
     <row r="239" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A239" s="2" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B239" s="2"/>
       <c r="C239" s="2"/>
@@ -4762,24 +4762,24 @@
     </row>
     <row r="240" spans="1:15" x14ac:dyDescent="0.25">
       <c r="J240" s="6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K240" s="6" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L240" s="14">
         <v>0</v>
       </c>
       <c r="M240" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="N240" s="6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="241" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A241" s="1" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J241" s="6"/>
       <c r="K241" s="6"/>
@@ -4789,1040 +4789,1040 @@
     </row>
     <row r="242" spans="1:15" x14ac:dyDescent="0.25">
       <c r="E242" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J242" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K242" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L242" s="12">
         <f>8/1000*(14/(1*14+3*2))*100</f>
         <v>0.55999999999999994</v>
       </c>
       <c r="M242" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="N242" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="O242" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="243" spans="1:15" x14ac:dyDescent="0.25">
       <c r="E243" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J243" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K243" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L243" s="12">
         <f>15/1000*(14/(1*14+3*2))*100</f>
         <v>1.0499999999999998</v>
       </c>
       <c r="M243" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O243" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="244" spans="1:15" x14ac:dyDescent="0.25">
       <c r="E244" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J244" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K244" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L244" s="12">
         <f>50/1000*(14/(1*14+3*2))*100</f>
         <v>3.4999999999999996</v>
       </c>
       <c r="M244" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O244" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="245" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A245" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B245" s="7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="246" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F246" t="s">
+        <v>140</v>
+      </c>
+      <c r="G246" t="s">
         <v>141</v>
       </c>
-      <c r="G246" t="s">
+      <c r="H246" t="s">
         <v>142</v>
       </c>
-      <c r="H246" t="s">
-        <v>143</v>
-      </c>
       <c r="I246" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J246" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K246" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L246">
         <v>33</v>
       </c>
       <c r="M246" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O246" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="247" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F247" t="s">
+        <v>140</v>
+      </c>
+      <c r="G247" t="s">
         <v>141</v>
       </c>
-      <c r="G247" t="s">
+      <c r="H247" t="s">
         <v>142</v>
       </c>
-      <c r="H247" t="s">
-        <v>143</v>
-      </c>
       <c r="I247" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="J247" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K247" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L247">
         <v>38</v>
       </c>
       <c r="M247" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O247" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="248" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F248" t="s">
+        <v>140</v>
+      </c>
+      <c r="G248" t="s">
         <v>141</v>
       </c>
-      <c r="G248" t="s">
+      <c r="H248" t="s">
         <v>142</v>
       </c>
-      <c r="H248" t="s">
-        <v>143</v>
-      </c>
       <c r="I248" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J248" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K248" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L248">
         <v>41</v>
       </c>
       <c r="M248" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O248" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="249" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F249" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G249" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H249" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I249" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J249" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K249" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L249">
         <v>32</v>
       </c>
       <c r="M249" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O249" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="250" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F250" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G250" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H250" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I250" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="J250" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K250" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L250">
         <v>39</v>
       </c>
       <c r="M250" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O250" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="251" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F251" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G251" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="H251" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="I251" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J251" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K251" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L251">
         <v>46</v>
       </c>
       <c r="M251" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O251" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="252" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F252" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H252" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I252" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J252" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K252" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L252">
         <v>32</v>
       </c>
       <c r="M252" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O252" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="253" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F253" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H253" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I253" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="J253" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K253" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L253">
         <v>38</v>
       </c>
       <c r="M253" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O253" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="254" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F254" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H254" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="I254" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J254" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K254" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L254">
         <v>47</v>
       </c>
       <c r="M254" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O254" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="255" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F255" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H255" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I255" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J255" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K255" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L255">
         <v>33</v>
       </c>
       <c r="M255" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O255" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="256" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F256" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H256" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I256" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="J256" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K256" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L256">
         <v>39</v>
       </c>
       <c r="M256" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O256" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="257" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F257" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="H257" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="I257" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J257" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K257" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L257">
         <v>47</v>
       </c>
       <c r="M257" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O257" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="258" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F258" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="I258" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J258" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K258" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L258">
         <v>32</v>
       </c>
       <c r="M258" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="N258" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="O258" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="259" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F259" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="I259" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="J259" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K259" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L259">
         <v>39</v>
       </c>
       <c r="M259" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="N259" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="O259" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="260" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F260" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="I260" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J260" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K260" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L260">
         <v>46</v>
       </c>
       <c r="M260" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="N260" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="O260" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="261" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F261" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="I261" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="J261" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K261" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L261">
         <v>14</v>
       </c>
       <c r="M261" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O261" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="262" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F262" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I262" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="J262" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K262" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L262">
         <v>43</v>
       </c>
       <c r="M262" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O262" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="263" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F263" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I263" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J263" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K263" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L263">
         <v>47</v>
       </c>
       <c r="M263" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O263" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="264" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F264" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I264" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="J264" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K264" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L264">
         <v>35</v>
       </c>
       <c r="M264" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O264" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="265" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F265" t="s">
+        <v>146</v>
+      </c>
+      <c r="H265" t="s">
         <v>147</v>
       </c>
-      <c r="H265" t="s">
-        <v>148</v>
-      </c>
       <c r="I265" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J265" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K265" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L265">
         <v>30</v>
       </c>
       <c r="M265" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O265" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="266" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F266" t="s">
+        <v>146</v>
+      </c>
+      <c r="H266" t="s">
         <v>147</v>
       </c>
-      <c r="H266" t="s">
-        <v>148</v>
-      </c>
       <c r="I266" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="J266" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K266" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L266">
         <v>35</v>
       </c>
       <c r="M266" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O266" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="267" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F267" t="s">
+        <v>146</v>
+      </c>
+      <c r="H267" t="s">
         <v>147</v>
       </c>
-      <c r="H267" t="s">
-        <v>148</v>
-      </c>
       <c r="I267" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J267" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K267" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L267">
         <v>48</v>
       </c>
       <c r="M267" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O267" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="268" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F268" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H268" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="I268" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J268" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K268" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L268">
         <v>29</v>
       </c>
       <c r="M268" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O268" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="269" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F269" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H269" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="I269" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="J269" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K269" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L269">
         <v>34</v>
       </c>
       <c r="M269" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O269" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="270" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F270" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H270" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="I270" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J270" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K270" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L270">
         <v>46</v>
       </c>
       <c r="M270" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O270" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="271" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F271" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H271" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I271" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J271" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K271" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L271">
         <v>29</v>
       </c>
       <c r="M271" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O271" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="272" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F272" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H272" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I272" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="J272" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K272" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L272">
         <v>35</v>
       </c>
       <c r="M272" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O272" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="273" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F273" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H273" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I273" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J273" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K273" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L273">
         <v>48</v>
       </c>
       <c r="M273" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O273" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="274" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F274" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H274" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="I274" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J274" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K274" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L274" s="13">
         <f>L265</f>
         <v>30</v>
       </c>
       <c r="M274" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="N274" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="O274" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="275" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F275" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H275" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="I275" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="J275" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K275" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L275" s="13">
         <f t="shared" ref="L275:L276" si="4">L266</f>
         <v>35</v>
       </c>
       <c r="M275" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="N275" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="O275" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="276" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F276" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="H276" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="I276" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J276" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K276" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L276" s="13">
         <f t="shared" si="4"/>
         <v>48</v>
       </c>
       <c r="M276" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="N276" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="O276" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="277" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F277" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I277" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J277" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K277" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L277">
         <v>29</v>
       </c>
       <c r="M277" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="N277" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O277" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="278" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F278" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I278" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="J278" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K278" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L278">
         <v>35</v>
       </c>
       <c r="M278" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="N278" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O278" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="279" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F279" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="I279" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J279" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K279" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L279">
         <v>44</v>
       </c>
       <c r="M279" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="N279" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O279" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="280" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F280" t="s">
+        <v>151</v>
+      </c>
+      <c r="G280" t="s">
         <v>152</v>
       </c>
-      <c r="G280" t="s">
-        <v>153</v>
-      </c>
       <c r="I280" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="J280" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K280" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L280">
         <v>41</v>
       </c>
       <c r="M280" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O280" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="281" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F281" t="s">
+        <v>151</v>
+      </c>
+      <c r="G281" t="s">
         <v>152</v>
       </c>
-      <c r="G281" t="s">
-        <v>153</v>
-      </c>
       <c r="I281" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J281" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K281" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="L281">
         <v>41</v>
       </c>
       <c r="M281" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O281" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="283" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A283" s="7" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="285" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A285" s="2" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B285" s="2"/>
       <c r="C285" s="2"/>
@@ -5841,145 +5841,145 @@
     </row>
     <row r="287" spans="1:15" x14ac:dyDescent="0.25">
       <c r="J287" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="K287" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="L287">
         <v>1</v>
       </c>
       <c r="M287" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="N287" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="O287" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="288" spans="1:15" x14ac:dyDescent="0.25">
       <c r="J288" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="K288" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="L288">
         <v>1</v>
       </c>
       <c r="M288" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="N288" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="O288" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="289" spans="6:15" x14ac:dyDescent="0.25">
       <c r="F289" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="I289" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="J289" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="K289" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="L289">
         <v>2</v>
       </c>
       <c r="M289" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="N289" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="O289" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="290" spans="6:15" x14ac:dyDescent="0.25">
       <c r="I290" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="J290" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="K290" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="L290">
         <v>1</v>
       </c>
       <c r="M290" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="N290" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="O290" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="291" spans="6:15" x14ac:dyDescent="0.25">
       <c r="J291" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="K291" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="L291">
         <v>1</v>
       </c>
       <c r="M291" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="N291" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="O291" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="292" spans="6:15" x14ac:dyDescent="0.25">
       <c r="J292" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="K292" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="L292">
         <v>1</v>
       </c>
       <c r="M292" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="N292" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="O292" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="294" spans="6:15" x14ac:dyDescent="0.25">
       <c r="J294" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="K294" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="L294">
         <v>13</v>
       </c>
       <c r="M294" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
   </sheetData>

</xml_diff>